<commit_message>
Update dashboard with light theme and forward-looking features
Changes:
- Switch to clean light theme (white background, subtle shadows)
- Projects now have ProjectType (Active/Planned) with Probability %
- New forward-looking visualizations:
  * Project Pipeline chart (Active vs Planned with FTE)
  * Aggregate Utilization Forecast (capacity vs demand over time)
  * Supply vs Demand Gap by skill
  * Available Resources for Staffing table with recommendations
  * Projects Needing Resources table with staffing gaps
- Updated metrics: Active Projects, Planned Projects (weighted FTE),
  Available Capacity, Overloaded resources
- Resource utilization heatmap shows who should go where
- Gantt chart distinguishes Active (green) vs Planned (blue) projects
- Support for partial chargeability across multiple projects
</commit_message>
<xml_diff>
--- a/resource_planning_data.xlsx
+++ b/resource_planning_data.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,6 +423,9 @@
       <c r="G1" t="str">
         <v>HoursPerWeek</v>
       </c>
+      <c r="H1" t="str">
+        <v>CostRate</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,6 +449,9 @@
       <c r="G2">
         <v>40</v>
       </c>
+      <c r="H2">
+        <v>150</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -469,6 +475,9 @@
       <c r="G3">
         <v>40</v>
       </c>
+      <c r="H3">
+        <v>160</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -492,6 +501,9 @@
       <c r="G4">
         <v>40</v>
       </c>
+      <c r="H4">
+        <v>175</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -515,6 +527,9 @@
       <c r="G5">
         <v>40</v>
       </c>
+      <c r="H5">
+        <v>140</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -538,6 +553,9 @@
       <c r="G6">
         <v>40</v>
       </c>
+      <c r="H6">
+        <v>155</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -561,6 +579,9 @@
       <c r="G7">
         <v>40</v>
       </c>
+      <c r="H7">
+        <v>145</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -584,6 +605,9 @@
       <c r="G8">
         <v>40</v>
       </c>
+      <c r="H8">
+        <v>165</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -607,6 +631,9 @@
       <c r="G9">
         <v>40</v>
       </c>
+      <c r="H9">
+        <v>130</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -625,10 +652,13 @@
         <v>Design</v>
       </c>
       <c r="F10" t="str">
-        <v>On Leave</v>
+        <v>Active</v>
       </c>
       <c r="G10">
         <v>40</v>
+      </c>
+      <c r="H10">
+        <v>140</v>
       </c>
     </row>
     <row r="11">
@@ -653,6 +683,9 @@
       <c r="G11">
         <v>40</v>
       </c>
+      <c r="H11">
+        <v>180</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -676,6 +709,9 @@
       <c r="G12">
         <v>40</v>
       </c>
+      <c r="H12">
+        <v>150</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -699,17 +735,98 @@
       <c r="G13">
         <v>40</v>
       </c>
+      <c r="H13">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>R013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Maria Santos</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Backend</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Microservices</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G14">
+        <v>40</v>
+      </c>
+      <c r="H14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>R014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Nathan Park</v>
+      </c>
+      <c r="C15" t="str">
+        <v>DevOps</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Kubernetes</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Infrastructure</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G15">
+        <v>40</v>
+      </c>
+      <c r="H15">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>R015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Olivia Kim</v>
+      </c>
+      <c r="C16" t="str">
+        <v>QA</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Performance</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Quality</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G16">
+        <v>40</v>
+      </c>
+      <c r="H16">
+        <v>135</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -722,21 +839,24 @@
         <v>Client</v>
       </c>
       <c r="D1" t="str">
-        <v>Status</v>
+        <v>ProjectType</v>
       </c>
       <c r="E1" t="str">
+        <v>Probability</v>
+      </c>
+      <c r="F1" t="str">
         <v>Priority</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>StartDate</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>EndDate</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Budget</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>RequiredFTE</v>
       </c>
     </row>
@@ -751,21 +871,24 @@
         <v>RetailCorp</v>
       </c>
       <c r="D2" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+      <c r="F2" t="str">
         <v>High</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>2025-01-15</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>2025-06-30</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>150000</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>4</v>
       </c>
     </row>
@@ -780,21 +903,24 @@
         <v>FinanceHub</v>
       </c>
       <c r="D3" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="E3" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3" t="str">
         <v>Critical</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>2025-02-01</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>2025-08-31</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>200000</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>5</v>
       </c>
     </row>
@@ -803,27 +929,30 @@
         <v>P003</v>
       </c>
       <c r="B4" t="str">
-        <v>Analytics Dashboard</v>
+        <v>CRM Integration</v>
       </c>
       <c r="C4" t="str">
-        <v>DataDriven Inc</v>
+        <v>SalesForce Plus</v>
       </c>
       <c r="D4" t="str">
-        <v>Planning</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Medium</v>
+        <v>Active</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
       </c>
       <c r="F4" t="str">
-        <v>2025-03-01</v>
+        <v>High</v>
       </c>
       <c r="G4" t="str">
-        <v>2025-07-15</v>
-      </c>
-      <c r="H4">
-        <v>80000</v>
+        <v>2025-01-01</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2025-05-31</v>
       </c>
       <c r="I4">
+        <v>120000</v>
+      </c>
+      <c r="J4">
         <v>3</v>
       </c>
     </row>
@@ -832,28 +961,31 @@
         <v>P004</v>
       </c>
       <c r="B5" t="str">
-        <v>CRM Integration</v>
+        <v>HR Portal</v>
       </c>
       <c r="C5" t="str">
-        <v>SalesForce Plus</v>
+        <v>Internal</v>
       </c>
       <c r="D5" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="E5" t="str">
-        <v>High</v>
+        <v>Active</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
       </c>
       <c r="F5" t="str">
-        <v>2025-01-01</v>
+        <v>Medium</v>
       </c>
       <c r="G5" t="str">
-        <v>2025-04-30</v>
-      </c>
-      <c r="H5">
-        <v>120000</v>
+        <v>2025-02-15</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2025-06-30</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>60000</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -861,28 +993,31 @@
         <v>P005</v>
       </c>
       <c r="B6" t="str">
-        <v>Cloud Migration</v>
+        <v>Analytics Dashboard</v>
       </c>
       <c r="C6" t="str">
-        <v>TechStart</v>
+        <v>DataDriven Inc</v>
       </c>
       <c r="D6" t="str">
-        <v>On Hold</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Low</v>
+        <v>Planned</v>
+      </c>
+      <c r="E6">
+        <v>85</v>
       </c>
       <c r="F6" t="str">
+        <v>High</v>
+      </c>
+      <c r="G6" t="str">
         <v>2025-04-01</v>
       </c>
-      <c r="G6" t="str">
-        <v>2025-09-30</v>
-      </c>
-      <c r="H6">
-        <v>250000</v>
+      <c r="H6" t="str">
+        <v>2025-08-15</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>80000</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -890,27 +1025,30 @@
         <v>P006</v>
       </c>
       <c r="B7" t="str">
-        <v>AI Chatbot</v>
+        <v>Cloud Migration</v>
       </c>
       <c r="C7" t="str">
-        <v>ServiceNow</v>
+        <v>TechStart</v>
       </c>
       <c r="D7" t="str">
-        <v>Planning</v>
-      </c>
-      <c r="E7" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="E7">
+        <v>70</v>
+      </c>
+      <c r="F7" t="str">
         <v>Medium</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>2025-05-01</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>2025-10-31</v>
       </c>
-      <c r="H7">
-        <v>180000</v>
-      </c>
       <c r="I7">
+        <v>250000</v>
+      </c>
+      <c r="J7">
         <v>4</v>
       </c>
     </row>
@@ -919,28 +1057,31 @@
         <v>P007</v>
       </c>
       <c r="B8" t="str">
-        <v>Inventory System</v>
+        <v>AI Chatbot</v>
       </c>
       <c r="C8" t="str">
-        <v>WarehousePro</v>
+        <v>ServiceNow</v>
       </c>
       <c r="D8" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="E8" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="E8">
+        <v>60</v>
+      </c>
+      <c r="F8" t="str">
         <v>Medium</v>
       </c>
-      <c r="F8" t="str">
-        <v>2024-10-01</v>
-      </c>
       <c r="G8" t="str">
-        <v>2025-01-31</v>
-      </c>
-      <c r="H8">
-        <v>90000</v>
+        <v>2025-06-01</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2025-11-30</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>180000</v>
+      </c>
+      <c r="J8">
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -948,40 +1089,139 @@
         <v>P008</v>
       </c>
       <c r="B9" t="str">
-        <v>HR Portal</v>
+        <v>Inventory System</v>
       </c>
       <c r="C9" t="str">
-        <v>Internal</v>
+        <v>WarehousePro</v>
       </c>
       <c r="D9" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="E9" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="E9">
+        <v>90</v>
+      </c>
+      <c r="F9" t="str">
         <v>High</v>
       </c>
-      <c r="F9" t="str">
-        <v>2025-02-15</v>
-      </c>
       <c r="G9" t="str">
-        <v>2025-05-31</v>
-      </c>
-      <c r="H9">
-        <v>60000</v>
+        <v>2025-04-15</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2025-07-31</v>
       </c>
       <c r="I9">
+        <v>90000</v>
+      </c>
+      <c r="J9">
         <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>P009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Payment Gateway</v>
+      </c>
+      <c r="C10" t="str">
+        <v>PaySecure</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="E10">
+        <v>75</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2025-05-15</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2025-09-30</v>
+      </c>
+      <c r="I10">
+        <v>140000</v>
+      </c>
+      <c r="J10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>P010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Customer Portal</v>
+      </c>
+      <c r="C11" t="str">
+        <v>RetailCorp</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="E11">
+        <v>50</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2025-07-01</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2025-12-31</v>
+      </c>
+      <c r="I11">
+        <v>100000</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>P011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Data Warehouse</v>
+      </c>
+      <c r="C12" t="str">
+        <v>DataDriven Inc</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="E12">
+        <v>40</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2025-08-01</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-01-31</v>
+      </c>
+      <c r="I12">
+        <v>200000</v>
+      </c>
+      <c r="J12">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:F106"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1002,9 +1242,6 @@
       <c r="F1" t="str">
         <v>Role</v>
       </c>
-      <c r="G1" t="str">
-        <v>HoursAllocated</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1020,13 +1257,10 @@
         <v>Jan-2025</v>
       </c>
       <c r="E2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F2" t="str">
         <v>Lead Developer</v>
-      </c>
-      <c r="G2">
-        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -1043,13 +1277,10 @@
         <v>Jan-2025</v>
       </c>
       <c r="E3">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F3" t="str">
         <v>Developer</v>
-      </c>
-      <c r="G3">
-        <v>80</v>
       </c>
     </row>
     <row r="4">
@@ -1066,13 +1297,10 @@
         <v>Feb-2025</v>
       </c>
       <c r="E4">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F4" t="str">
         <v>Lead Developer</v>
-      </c>
-      <c r="G4">
-        <v>112</v>
       </c>
     </row>
     <row r="5">
@@ -1089,13 +1317,10 @@
         <v>Feb-2025</v>
       </c>
       <c r="E5">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F5" t="str">
         <v>Developer</v>
-      </c>
-      <c r="G5">
-        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -1112,13 +1337,10 @@
         <v>Mar-2025</v>
       </c>
       <c r="E6">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F6" t="str">
         <v>Lead Developer</v>
-      </c>
-      <c r="G6">
-        <v>128</v>
       </c>
     </row>
     <row r="7">
@@ -1129,19 +1351,16 @@
         <v>R001</v>
       </c>
       <c r="C7" t="str">
-        <v>P008</v>
+        <v>P004</v>
       </c>
       <c r="D7" t="str">
         <v>Mar-2025</v>
       </c>
       <c r="E7">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F7" t="str">
         <v>Developer</v>
-      </c>
-      <c r="G7">
-        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -1149,22 +1368,19 @@
         <v>A007</v>
       </c>
       <c r="B8" t="str">
-        <v>R002</v>
+        <v>R001</v>
       </c>
       <c r="C8" t="str">
         <v>P001</v>
       </c>
       <c r="D8" t="str">
-        <v>Jan-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E8">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F8" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G8">
-        <v>80</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="9">
@@ -1172,22 +1388,19 @@
         <v>A008</v>
       </c>
       <c r="B9" t="str">
-        <v>R002</v>
+        <v>R001</v>
       </c>
       <c r="C9" t="str">
-        <v>P002</v>
+        <v>P005</v>
       </c>
       <c r="D9" t="str">
-        <v>Jan-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E9">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F9" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G9">
-        <v>64</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="10">
@@ -1195,22 +1408,19 @@
         <v>A009</v>
       </c>
       <c r="B10" t="str">
-        <v>R002</v>
+        <v>R001</v>
       </c>
       <c r="C10" t="str">
-        <v>P004</v>
+        <v>P001</v>
       </c>
       <c r="D10" t="str">
-        <v>Jan-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E10">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F10" t="str">
-        <v>Developer</v>
-      </c>
-      <c r="G10">
-        <v>48</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="11">
@@ -1218,22 +1428,19 @@
         <v>A010</v>
       </c>
       <c r="B11" t="str">
-        <v>R002</v>
+        <v>R001</v>
       </c>
       <c r="C11" t="str">
-        <v>P001</v>
+        <v>P005</v>
       </c>
       <c r="D11" t="str">
-        <v>Feb-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E11">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F11" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G11">
-        <v>96</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="12">
@@ -1241,22 +1448,19 @@
         <v>A011</v>
       </c>
       <c r="B12" t="str">
-        <v>R002</v>
+        <v>R001</v>
       </c>
       <c r="C12" t="str">
-        <v>P002</v>
+        <v>P001</v>
       </c>
       <c r="D12" t="str">
-        <v>Feb-2025</v>
+        <v>Jun-2025</v>
       </c>
       <c r="E12">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F12" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G12">
-        <v>80</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="13">
@@ -1264,22 +1468,19 @@
         <v>A012</v>
       </c>
       <c r="B13" t="str">
-        <v>R002</v>
+        <v>R001</v>
       </c>
       <c r="C13" t="str">
-        <v>P001</v>
+        <v>P005</v>
       </c>
       <c r="D13" t="str">
-        <v>Mar-2025</v>
+        <v>Jun-2025</v>
       </c>
       <c r="E13">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F13" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G13">
-        <v>64</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="14">
@@ -1290,19 +1491,16 @@
         <v>R002</v>
       </c>
       <c r="C14" t="str">
-        <v>P002</v>
+        <v>P001</v>
       </c>
       <c r="D14" t="str">
-        <v>Mar-2025</v>
+        <v>Jan-2025</v>
       </c>
       <c r="E14">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F14" t="str">
         <v>Backend Developer</v>
-      </c>
-      <c r="G14">
-        <v>96</v>
       </c>
     </row>
     <row r="15">
@@ -1310,22 +1508,19 @@
         <v>A014</v>
       </c>
       <c r="B15" t="str">
-        <v>R003</v>
+        <v>R002</v>
       </c>
       <c r="C15" t="str">
-        <v>P003</v>
+        <v>P002</v>
       </c>
       <c r="D15" t="str">
         <v>Jan-2025</v>
       </c>
       <c r="E15">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F15" t="str">
-        <v>Data Analyst</v>
-      </c>
-      <c r="G15">
-        <v>32</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="16">
@@ -1333,22 +1528,19 @@
         <v>A015</v>
       </c>
       <c r="B16" t="str">
-        <v>R003</v>
+        <v>R002</v>
       </c>
       <c r="C16" t="str">
         <v>P003</v>
       </c>
       <c r="D16" t="str">
-        <v>Feb-2025</v>
+        <v>Jan-2025</v>
       </c>
       <c r="E16">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F16" t="str">
-        <v>Data Analyst</v>
-      </c>
-      <c r="G16">
-        <v>48</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="17">
@@ -1356,22 +1548,19 @@
         <v>A016</v>
       </c>
       <c r="B17" t="str">
-        <v>R003</v>
+        <v>R002</v>
       </c>
       <c r="C17" t="str">
-        <v>P003</v>
+        <v>P001</v>
       </c>
       <c r="D17" t="str">
-        <v>Mar-2025</v>
+        <v>Feb-2025</v>
       </c>
       <c r="E17">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F17" t="str">
-        <v>Data Analyst</v>
-      </c>
-      <c r="G17">
-        <v>64</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="18">
@@ -1379,22 +1568,19 @@
         <v>A017</v>
       </c>
       <c r="B18" t="str">
-        <v>R003</v>
+        <v>R002</v>
       </c>
       <c r="C18" t="str">
-        <v>P006</v>
+        <v>P002</v>
       </c>
       <c r="D18" t="str">
-        <v>Mar-2025</v>
+        <v>Feb-2025</v>
       </c>
       <c r="E18">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F18" t="str">
-        <v>ML Engineer</v>
-      </c>
-      <c r="G18">
-        <v>32</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="19">
@@ -1402,22 +1588,19 @@
         <v>A018</v>
       </c>
       <c r="B19" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C19" t="str">
         <v>P001</v>
       </c>
       <c r="D19" t="str">
-        <v>Jan-2025</v>
+        <v>Mar-2025</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F19" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G19">
-        <v>48</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="20">
@@ -1425,22 +1608,19 @@
         <v>A019</v>
       </c>
       <c r="B20" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C20" t="str">
         <v>P002</v>
       </c>
       <c r="D20" t="str">
-        <v>Jan-2025</v>
+        <v>Mar-2025</v>
       </c>
       <c r="E20">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F20" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G20">
-        <v>64</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="21">
@@ -1448,22 +1628,19 @@
         <v>A020</v>
       </c>
       <c r="B21" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C21" t="str">
-        <v>P001</v>
+        <v>P002</v>
       </c>
       <c r="D21" t="str">
-        <v>Feb-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E21">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F21" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G21">
-        <v>40</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="22">
@@ -1471,22 +1648,19 @@
         <v>A021</v>
       </c>
       <c r="B22" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C22" t="str">
-        <v>P002</v>
+        <v>P005</v>
       </c>
       <c r="D22" t="str">
-        <v>Feb-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E22">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="F22" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G22">
-        <v>72</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="23">
@@ -1494,22 +1668,19 @@
         <v>A022</v>
       </c>
       <c r="B23" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C23" t="str">
-        <v>P003</v>
+        <v>P002</v>
       </c>
       <c r="D23" t="str">
-        <v>Feb-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E23">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F23" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G23">
-        <v>32</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="24">
@@ -1517,22 +1688,19 @@
         <v>A023</v>
       </c>
       <c r="B24" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C24" t="str">
-        <v>P001</v>
+        <v>P006</v>
       </c>
       <c r="D24" t="str">
-        <v>Mar-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E24">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F24" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G24">
-        <v>32</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="25">
@@ -1540,22 +1708,19 @@
         <v>A024</v>
       </c>
       <c r="B25" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C25" t="str">
         <v>P002</v>
       </c>
       <c r="D25" t="str">
-        <v>Mar-2025</v>
+        <v>Jun-2025</v>
       </c>
       <c r="E25">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F25" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G25">
-        <v>80</v>
+        <v>Backend Developer</v>
       </c>
     </row>
     <row r="26">
@@ -1563,22 +1728,19 @@
         <v>A025</v>
       </c>
       <c r="B26" t="str">
-        <v>R004</v>
+        <v>R002</v>
       </c>
       <c r="C26" t="str">
-        <v>P003</v>
+        <v>P006</v>
       </c>
       <c r="D26" t="str">
-        <v>Mar-2025</v>
+        <v>Jun-2025</v>
       </c>
       <c r="E26">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F26" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="G26">
-        <v>48</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="27">
@@ -1586,22 +1748,19 @@
         <v>A026</v>
       </c>
       <c r="B27" t="str">
-        <v>R005</v>
+        <v>R003</v>
       </c>
       <c r="C27" t="str">
-        <v>P004</v>
+        <v>P003</v>
       </c>
       <c r="D27" t="str">
         <v>Jan-2025</v>
       </c>
       <c r="E27">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="F27" t="str">
-        <v>Lead Developer</v>
-      </c>
-      <c r="G27">
-        <v>128</v>
+        <v>Data Analyst</v>
       </c>
     </row>
     <row r="28">
@@ -1609,22 +1768,19 @@
         <v>A027</v>
       </c>
       <c r="B28" t="str">
-        <v>R005</v>
+        <v>R003</v>
       </c>
       <c r="C28" t="str">
-        <v>P004</v>
+        <v>P003</v>
       </c>
       <c r="D28" t="str">
         <v>Feb-2025</v>
       </c>
       <c r="E28">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="F28" t="str">
-        <v>Lead Developer</v>
-      </c>
-      <c r="G28">
-        <v>144</v>
+        <v>Data Analyst</v>
       </c>
     </row>
     <row r="29">
@@ -1632,22 +1788,19 @@
         <v>A028</v>
       </c>
       <c r="B29" t="str">
-        <v>R005</v>
+        <v>R003</v>
       </c>
       <c r="C29" t="str">
-        <v>P004</v>
+        <v>P003</v>
       </c>
       <c r="D29" t="str">
         <v>Mar-2025</v>
       </c>
       <c r="E29">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F29" t="str">
-        <v>Lead Developer</v>
-      </c>
-      <c r="G29">
-        <v>112</v>
+        <v>Data Analyst</v>
       </c>
     </row>
     <row r="30">
@@ -1655,22 +1808,19 @@
         <v>A029</v>
       </c>
       <c r="B30" t="str">
-        <v>R005</v>
+        <v>R003</v>
       </c>
       <c r="C30" t="str">
-        <v>P008</v>
+        <v>P005</v>
       </c>
       <c r="D30" t="str">
-        <v>Mar-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E30">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F30" t="str">
-        <v>Developer</v>
-      </c>
-      <c r="G30">
-        <v>48</v>
+        <v>Lead Data Scientist</v>
       </c>
     </row>
     <row r="31">
@@ -1678,22 +1828,19 @@
         <v>A030</v>
       </c>
       <c r="B31" t="str">
-        <v>R006</v>
+        <v>R003</v>
       </c>
       <c r="C31" t="str">
-        <v>P008</v>
+        <v>P005</v>
       </c>
       <c r="D31" t="str">
-        <v>Feb-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E31">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="F31" t="str">
-        <v>Frontend Developer</v>
-      </c>
-      <c r="G31">
-        <v>64</v>
+        <v>Lead Data Scientist</v>
       </c>
     </row>
     <row r="32">
@@ -1701,22 +1848,19 @@
         <v>A031</v>
       </c>
       <c r="B32" t="str">
-        <v>R006</v>
+        <v>R003</v>
       </c>
       <c r="C32" t="str">
-        <v>P008</v>
+        <v>P005</v>
       </c>
       <c r="D32" t="str">
-        <v>Mar-2025</v>
+        <v>Jun-2025</v>
       </c>
       <c r="E32">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="F32" t="str">
-        <v>Frontend Developer</v>
-      </c>
-      <c r="G32">
-        <v>80</v>
+        <v>Lead Data Scientist</v>
       </c>
     </row>
     <row r="33">
@@ -1724,22 +1868,19 @@
         <v>A032</v>
       </c>
       <c r="B33" t="str">
-        <v>R007</v>
+        <v>R003</v>
       </c>
       <c r="C33" t="str">
-        <v>P005</v>
+        <v>P007</v>
       </c>
       <c r="D33" t="str">
-        <v>Jan-2025</v>
+        <v>Jun-2025</v>
       </c>
       <c r="E33">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F33" t="str">
-        <v>DevOps Engineer</v>
-      </c>
-      <c r="G33">
-        <v>48</v>
+        <v>ML Engineer</v>
       </c>
     </row>
     <row r="34">
@@ -1747,22 +1888,19 @@
         <v>A033</v>
       </c>
       <c r="B34" t="str">
-        <v>R007</v>
+        <v>R004</v>
       </c>
       <c r="C34" t="str">
-        <v>P002</v>
+        <v>P001</v>
       </c>
       <c r="D34" t="str">
         <v>Jan-2025</v>
       </c>
       <c r="E34">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F34" t="str">
-        <v>DevOps Engineer</v>
-      </c>
-      <c r="G34">
-        <v>32</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="35">
@@ -1770,22 +1908,19 @@
         <v>A034</v>
       </c>
       <c r="B35" t="str">
-        <v>R007</v>
+        <v>R004</v>
       </c>
       <c r="C35" t="str">
-        <v>P005</v>
+        <v>P002</v>
       </c>
       <c r="D35" t="str">
-        <v>Feb-2025</v>
+        <v>Jan-2025</v>
       </c>
       <c r="E35">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F35" t="str">
-        <v>DevOps Engineer</v>
-      </c>
-      <c r="G35">
-        <v>40</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="36">
@@ -1793,22 +1928,19 @@
         <v>A035</v>
       </c>
       <c r="B36" t="str">
-        <v>R007</v>
+        <v>R004</v>
       </c>
       <c r="C36" t="str">
-        <v>P002</v>
+        <v>P003</v>
       </c>
       <c r="D36" t="str">
-        <v>Feb-2025</v>
+        <v>Jan-2025</v>
       </c>
       <c r="E36">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F36" t="str">
-        <v>DevOps Engineer</v>
-      </c>
-      <c r="G36">
-        <v>48</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="37">
@@ -1816,22 +1948,19 @@
         <v>A036</v>
       </c>
       <c r="B37" t="str">
-        <v>R007</v>
+        <v>R004</v>
       </c>
       <c r="C37" t="str">
-        <v>P002</v>
+        <v>P001</v>
       </c>
       <c r="D37" t="str">
-        <v>Mar-2025</v>
+        <v>Feb-2025</v>
       </c>
       <c r="E37">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F37" t="str">
-        <v>DevOps Engineer</v>
-      </c>
-      <c r="G37">
-        <v>64</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="38">
@@ -1839,22 +1968,19 @@
         <v>A037</v>
       </c>
       <c r="B38" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C38" t="str">
-        <v>P001</v>
+        <v>P002</v>
       </c>
       <c r="D38" t="str">
-        <v>Jan-2025</v>
+        <v>Feb-2025</v>
       </c>
       <c r="E38">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F38" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G38">
-        <v>64</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="39">
@@ -1862,22 +1988,19 @@
         <v>A038</v>
       </c>
       <c r="B39" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C39" t="str">
-        <v>P002</v>
+        <v>P003</v>
       </c>
       <c r="D39" t="str">
-        <v>Jan-2025</v>
+        <v>Feb-2025</v>
       </c>
       <c r="E39">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F39" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G39">
-        <v>48</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="40">
@@ -1885,22 +2008,19 @@
         <v>A039</v>
       </c>
       <c r="B40" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C40" t="str">
-        <v>P001</v>
+        <v>P004</v>
       </c>
       <c r="D40" t="str">
         <v>Feb-2025</v>
       </c>
       <c r="E40">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F40" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G40">
-        <v>80</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="41">
@@ -1908,22 +2028,19 @@
         <v>A040</v>
       </c>
       <c r="B41" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C41" t="str">
-        <v>P002</v>
+        <v>P001</v>
       </c>
       <c r="D41" t="str">
-        <v>Feb-2025</v>
+        <v>Mar-2025</v>
       </c>
       <c r="E41">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F41" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G41">
-        <v>64</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="42">
@@ -1931,22 +2048,19 @@
         <v>A041</v>
       </c>
       <c r="B42" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C42" t="str">
-        <v>P004</v>
+        <v>P002</v>
       </c>
       <c r="D42" t="str">
-        <v>Feb-2025</v>
+        <v>Mar-2025</v>
       </c>
       <c r="E42">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F42" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G42">
-        <v>40</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="43">
@@ -1954,22 +2068,19 @@
         <v>A042</v>
       </c>
       <c r="B43" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C43" t="str">
-        <v>P001</v>
+        <v>P004</v>
       </c>
       <c r="D43" t="str">
         <v>Mar-2025</v>
       </c>
       <c r="E43">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F43" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G43">
-        <v>96</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="44">
@@ -1977,22 +2088,19 @@
         <v>A043</v>
       </c>
       <c r="B44" t="str">
-        <v>R008</v>
+        <v>R004</v>
       </c>
       <c r="C44" t="str">
-        <v>P002</v>
+        <v>P005</v>
       </c>
       <c r="D44" t="str">
-        <v>Mar-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E44">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F44" t="str">
-        <v>QA Engineer</v>
-      </c>
-      <c r="G44">
-        <v>80</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="45">
@@ -2000,22 +2108,19 @@
         <v>A044</v>
       </c>
       <c r="B45" t="str">
-        <v>R010</v>
+        <v>R004</v>
       </c>
       <c r="C45" t="str">
-        <v>P006</v>
+        <v>P002</v>
       </c>
       <c r="D45" t="str">
-        <v>Jan-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E45">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F45" t="str">
-        <v>ML Engineer</v>
-      </c>
-      <c r="G45">
-        <v>32</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="46">
@@ -2023,22 +2128,19 @@
         <v>A045</v>
       </c>
       <c r="B46" t="str">
-        <v>R010</v>
+        <v>R004</v>
       </c>
       <c r="C46" t="str">
-        <v>P003</v>
+        <v>P004</v>
       </c>
       <c r="D46" t="str">
-        <v>Feb-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E46">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F46" t="str">
-        <v>Data Scientist</v>
-      </c>
-      <c r="G46">
-        <v>80</v>
+        <v>Project Manager</v>
       </c>
     </row>
     <row r="47">
@@ -2046,22 +2148,19 @@
         <v>A046</v>
       </c>
       <c r="B47" t="str">
-        <v>R010</v>
+        <v>R005</v>
       </c>
       <c r="C47" t="str">
-        <v>P006</v>
+        <v>P003</v>
       </c>
       <c r="D47" t="str">
-        <v>Feb-2025</v>
+        <v>Jan-2025</v>
       </c>
       <c r="E47">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="F47" t="str">
-        <v>ML Engineer</v>
-      </c>
-      <c r="G47">
-        <v>48</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="48">
@@ -2069,22 +2168,19 @@
         <v>A047</v>
       </c>
       <c r="B48" t="str">
-        <v>R010</v>
+        <v>R005</v>
       </c>
       <c r="C48" t="str">
         <v>P003</v>
       </c>
       <c r="D48" t="str">
-        <v>Mar-2025</v>
+        <v>Feb-2025</v>
       </c>
       <c r="E48">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F48" t="str">
-        <v>Data Scientist</v>
-      </c>
-      <c r="G48">
-        <v>96</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="49">
@@ -2092,22 +2188,19 @@
         <v>A048</v>
       </c>
       <c r="B49" t="str">
-        <v>R010</v>
+        <v>R005</v>
       </c>
       <c r="C49" t="str">
-        <v>P006</v>
+        <v>P003</v>
       </c>
       <c r="D49" t="str">
         <v>Mar-2025</v>
       </c>
       <c r="E49">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F49" t="str">
-        <v>ML Engineer</v>
-      </c>
-      <c r="G49">
-        <v>64</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="50">
@@ -2115,22 +2208,19 @@
         <v>A049</v>
       </c>
       <c r="B50" t="str">
-        <v>R011</v>
+        <v>R005</v>
       </c>
       <c r="C50" t="str">
-        <v>P008</v>
+        <v>P003</v>
       </c>
       <c r="D50" t="str">
-        <v>Feb-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E50">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="F50" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G50">
-        <v>48</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="51">
@@ -2138,22 +2228,19 @@
         <v>A050</v>
       </c>
       <c r="B51" t="str">
-        <v>R011</v>
+        <v>R005</v>
       </c>
       <c r="C51" t="str">
-        <v>P008</v>
+        <v>P004</v>
       </c>
       <c r="D51" t="str">
-        <v>Mar-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E51">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F51" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="G51">
-        <v>64</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="52">
@@ -2161,22 +2248,19 @@
         <v>A051</v>
       </c>
       <c r="B52" t="str">
-        <v>R012</v>
+        <v>R005</v>
       </c>
       <c r="C52" t="str">
-        <v>P001</v>
+        <v>P003</v>
       </c>
       <c r="D52" t="str">
-        <v>Jan-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E52">
         <v>50</v>
       </c>
       <c r="F52" t="str">
-        <v>Frontend Developer</v>
-      </c>
-      <c r="G52">
-        <v>80</v>
+        <v>Lead Developer</v>
       </c>
     </row>
     <row r="53">
@@ -2184,22 +2268,19 @@
         <v>A052</v>
       </c>
       <c r="B53" t="str">
-        <v>R012</v>
+        <v>R005</v>
       </c>
       <c r="C53" t="str">
-        <v>P001</v>
+        <v>P009</v>
       </c>
       <c r="D53" t="str">
-        <v>Feb-2025</v>
+        <v>May-2025</v>
       </c>
       <c r="E53">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F53" t="str">
-        <v>Frontend Developer</v>
-      </c>
-      <c r="G53">
-        <v>96</v>
+        <v>Developer</v>
       </c>
     </row>
     <row r="54">
@@ -2207,22 +2288,19 @@
         <v>A053</v>
       </c>
       <c r="B54" t="str">
-        <v>R012</v>
+        <v>R006</v>
       </c>
       <c r="C54" t="str">
-        <v>P002</v>
+        <v>P004</v>
       </c>
       <c r="D54" t="str">
         <v>Feb-2025</v>
       </c>
       <c r="E54">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F54" t="str">
         <v>Frontend Developer</v>
-      </c>
-      <c r="G54">
-        <v>48</v>
       </c>
     </row>
     <row r="55">
@@ -2230,22 +2308,19 @@
         <v>A054</v>
       </c>
       <c r="B55" t="str">
-        <v>R012</v>
+        <v>R006</v>
       </c>
       <c r="C55" t="str">
-        <v>P001</v>
+        <v>P004</v>
       </c>
       <c r="D55" t="str">
         <v>Mar-2025</v>
       </c>
       <c r="E55">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F55" t="str">
         <v>Frontend Developer</v>
-      </c>
-      <c r="G55">
-        <v>80</v>
       </c>
     </row>
     <row r="56">
@@ -2253,27 +2328,1024 @@
         <v>A055</v>
       </c>
       <c r="B56" t="str">
-        <v>R012</v>
+        <v>R006</v>
       </c>
       <c r="C56" t="str">
-        <v>P002</v>
+        <v>P004</v>
       </c>
       <c r="D56" t="str">
-        <v>Mar-2025</v>
+        <v>Apr-2025</v>
       </c>
       <c r="E56">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F56" t="str">
         <v>Frontend Developer</v>
       </c>
-      <c r="G56">
-        <v>64</v>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>A056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>R006</v>
+      </c>
+      <c r="C57" t="str">
+        <v>P008</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Apr-2025</v>
+      </c>
+      <c r="E57">
+        <v>30</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Developer</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>A057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>R006</v>
+      </c>
+      <c r="C58" t="str">
+        <v>P004</v>
+      </c>
+      <c r="D58" t="str">
+        <v>May-2025</v>
+      </c>
+      <c r="E58">
+        <v>40</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Frontend Developer</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>A058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>R006</v>
+      </c>
+      <c r="C59" t="str">
+        <v>P008</v>
+      </c>
+      <c r="D59" t="str">
+        <v>May-2025</v>
+      </c>
+      <c r="E59">
+        <v>40</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Developer</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>A059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C60" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E60">
+        <v>30</v>
+      </c>
+      <c r="F60" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>A060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C61" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E61">
+        <v>20</v>
+      </c>
+      <c r="F61" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>A061</v>
+      </c>
+      <c r="B62" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C62" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E62">
+        <v>40</v>
+      </c>
+      <c r="F62" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>A062</v>
+      </c>
+      <c r="B63" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C63" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E63">
+        <v>20</v>
+      </c>
+      <c r="F63" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>A063</v>
+      </c>
+      <c r="B64" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C64" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E64">
+        <v>50</v>
+      </c>
+      <c r="F64" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>A064</v>
+      </c>
+      <c r="B65" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C65" t="str">
+        <v>P006</v>
+      </c>
+      <c r="D65" t="str">
+        <v>May-2025</v>
+      </c>
+      <c r="E65">
+        <v>60</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Lead DevOps</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>A065</v>
+      </c>
+      <c r="B66" t="str">
+        <v>R007</v>
+      </c>
+      <c r="C66" t="str">
+        <v>P006</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Jun-2025</v>
+      </c>
+      <c r="E66">
+        <v>80</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Lead DevOps</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>A066</v>
+      </c>
+      <c r="B67" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C67" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E67">
+        <v>30</v>
+      </c>
+      <c r="F67" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>A067</v>
+      </c>
+      <c r="B68" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C68" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E68">
+        <v>30</v>
+      </c>
+      <c r="F68" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>A068</v>
+      </c>
+      <c r="B69" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C69" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E69">
+        <v>40</v>
+      </c>
+      <c r="F69" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>A069</v>
+      </c>
+      <c r="B70" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C70" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E70">
+        <v>30</v>
+      </c>
+      <c r="F70" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>A070</v>
+      </c>
+      <c r="B71" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C71" t="str">
+        <v>P003</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E71">
+        <v>20</v>
+      </c>
+      <c r="F71" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>A071</v>
+      </c>
+      <c r="B72" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C72" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E72">
+        <v>50</v>
+      </c>
+      <c r="F72" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>A072</v>
+      </c>
+      <c r="B73" t="str">
+        <v>R008</v>
+      </c>
+      <c r="C73" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E73">
+        <v>40</v>
+      </c>
+      <c r="F73" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>A073</v>
+      </c>
+      <c r="B74" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C74" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E74">
+        <v>40</v>
+      </c>
+      <c r="F74" t="str">
+        <v>UI Designer</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>A074</v>
+      </c>
+      <c r="B75" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C75" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E75">
+        <v>30</v>
+      </c>
+      <c r="F75" t="str">
+        <v>UX Designer</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>A075</v>
+      </c>
+      <c r="B76" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C76" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E76">
+        <v>30</v>
+      </c>
+      <c r="F76" t="str">
+        <v>UI Designer</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>A076</v>
+      </c>
+      <c r="B77" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C77" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E77">
+        <v>40</v>
+      </c>
+      <c r="F77" t="str">
+        <v>UX Designer</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>A077</v>
+      </c>
+      <c r="B78" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C78" t="str">
+        <v>P004</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E78">
+        <v>20</v>
+      </c>
+      <c r="F78" t="str">
+        <v>UI Designer</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>A078</v>
+      </c>
+      <c r="B79" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C79" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E79">
+        <v>50</v>
+      </c>
+      <c r="F79" t="str">
+        <v>UX Designer</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>A079</v>
+      </c>
+      <c r="B80" t="str">
+        <v>R009</v>
+      </c>
+      <c r="C80" t="str">
+        <v>P004</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E80">
+        <v>30</v>
+      </c>
+      <c r="F80" t="str">
+        <v>UI Designer</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>A080</v>
+      </c>
+      <c r="B81" t="str">
+        <v>R010</v>
+      </c>
+      <c r="C81" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E81">
+        <v>30</v>
+      </c>
+      <c r="F81" t="str">
+        <v>ML Engineer</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>A081</v>
+      </c>
+      <c r="B82" t="str">
+        <v>R010</v>
+      </c>
+      <c r="C82" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E82">
+        <v>40</v>
+      </c>
+      <c r="F82" t="str">
+        <v>ML Engineer</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>A082</v>
+      </c>
+      <c r="B83" t="str">
+        <v>R010</v>
+      </c>
+      <c r="C83" t="str">
+        <v>P007</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Jun-2025</v>
+      </c>
+      <c r="E83">
+        <v>50</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Lead ML Engineer</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>A083</v>
+      </c>
+      <c r="B84" t="str">
+        <v>R010</v>
+      </c>
+      <c r="C84" t="str">
+        <v>P005</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Apr-2025</v>
+      </c>
+      <c r="E84">
+        <v>30</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Data Scientist</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>A084</v>
+      </c>
+      <c r="B85" t="str">
+        <v>R010</v>
+      </c>
+      <c r="C85" t="str">
+        <v>P005</v>
+      </c>
+      <c r="D85" t="str">
+        <v>May-2025</v>
+      </c>
+      <c r="E85">
+        <v>40</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Data Scientist</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>A085</v>
+      </c>
+      <c r="B86" t="str">
+        <v>R011</v>
+      </c>
+      <c r="C86" t="str">
+        <v>P004</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E86">
+        <v>30</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Backend Developer</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>A086</v>
+      </c>
+      <c r="B87" t="str">
+        <v>R011</v>
+      </c>
+      <c r="C87" t="str">
+        <v>P004</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Apr-2025</v>
+      </c>
+      <c r="E87">
+        <v>40</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Backend Developer</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>A087</v>
+      </c>
+      <c r="B88" t="str">
+        <v>R011</v>
+      </c>
+      <c r="C88" t="str">
+        <v>P008</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Apr-2025</v>
+      </c>
+      <c r="E88">
+        <v>20</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Developer</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>A088</v>
+      </c>
+      <c r="B89" t="str">
+        <v>R012</v>
+      </c>
+      <c r="C89" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E89">
+        <v>50</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Frontend Developer</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>A089</v>
+      </c>
+      <c r="B90" t="str">
+        <v>R012</v>
+      </c>
+      <c r="C90" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E90">
+        <v>60</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Frontend Developer</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>A090</v>
+      </c>
+      <c r="B91" t="str">
+        <v>R012</v>
+      </c>
+      <c r="C91" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E91">
+        <v>30</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Frontend Developer</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>A091</v>
+      </c>
+      <c r="B92" t="str">
+        <v>R012</v>
+      </c>
+      <c r="C92" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E92">
+        <v>50</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Frontend Developer</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>A092</v>
+      </c>
+      <c r="B93" t="str">
+        <v>R012</v>
+      </c>
+      <c r="C93" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E93">
+        <v>40</v>
+      </c>
+      <c r="F93" t="str">
+        <v>Frontend Developer</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>A093</v>
+      </c>
+      <c r="B94" t="str">
+        <v>R013</v>
+      </c>
+      <c r="C94" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E94">
+        <v>60</v>
+      </c>
+      <c r="F94" t="str">
+        <v>Backend Developer</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>A094</v>
+      </c>
+      <c r="B95" t="str">
+        <v>R013</v>
+      </c>
+      <c r="C95" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E95">
+        <v>70</v>
+      </c>
+      <c r="F95" t="str">
+        <v>Backend Developer</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>A095</v>
+      </c>
+      <c r="B96" t="str">
+        <v>R013</v>
+      </c>
+      <c r="C96" t="str">
+        <v>P002</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E96">
+        <v>60</v>
+      </c>
+      <c r="F96" t="str">
+        <v>Backend Developer</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>A096</v>
+      </c>
+      <c r="B97" t="str">
+        <v>R013</v>
+      </c>
+      <c r="C97" t="str">
+        <v>P009</v>
+      </c>
+      <c r="D97" t="str">
+        <v>May-2025</v>
+      </c>
+      <c r="E97">
+        <v>50</v>
+      </c>
+      <c r="F97" t="str">
+        <v>Developer</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>A097</v>
+      </c>
+      <c r="B98" t="str">
+        <v>R014</v>
+      </c>
+      <c r="C98" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E98">
+        <v>30</v>
+      </c>
+      <c r="F98" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>A098</v>
+      </c>
+      <c r="B99" t="str">
+        <v>R014</v>
+      </c>
+      <c r="C99" t="str">
+        <v>P003</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E99">
+        <v>30</v>
+      </c>
+      <c r="F99" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>A099</v>
+      </c>
+      <c r="B100" t="str">
+        <v>R014</v>
+      </c>
+      <c r="C100" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E100">
+        <v>30</v>
+      </c>
+      <c r="F100" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>A100</v>
+      </c>
+      <c r="B101" t="str">
+        <v>R014</v>
+      </c>
+      <c r="C101" t="str">
+        <v>P003</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E101">
+        <v>40</v>
+      </c>
+      <c r="F101" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>A101</v>
+      </c>
+      <c r="B102" t="str">
+        <v>R014</v>
+      </c>
+      <c r="C102" t="str">
+        <v>P006</v>
+      </c>
+      <c r="D102" t="str">
+        <v>May-2025</v>
+      </c>
+      <c r="E102">
+        <v>50</v>
+      </c>
+      <c r="F102" t="str">
+        <v>DevOps Engineer</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>A102</v>
+      </c>
+      <c r="B103" t="str">
+        <v>R015</v>
+      </c>
+      <c r="C103" t="str">
+        <v>P003</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Jan-2025</v>
+      </c>
+      <c r="E103">
+        <v>40</v>
+      </c>
+      <c r="F103" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>A103</v>
+      </c>
+      <c r="B104" t="str">
+        <v>R015</v>
+      </c>
+      <c r="C104" t="str">
+        <v>P003</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Feb-2025</v>
+      </c>
+      <c r="E104">
+        <v>50</v>
+      </c>
+      <c r="F104" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>A104</v>
+      </c>
+      <c r="B105" t="str">
+        <v>R015</v>
+      </c>
+      <c r="C105" t="str">
+        <v>P003</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E105">
+        <v>40</v>
+      </c>
+      <c r="F105" t="str">
+        <v>QA Engineer</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>A105</v>
+      </c>
+      <c r="B106" t="str">
+        <v>R015</v>
+      </c>
+      <c r="C106" t="str">
+        <v>P004</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Mar-2025</v>
+      </c>
+      <c r="E106">
+        <v>30</v>
+      </c>
+      <c r="F106" t="str">
+        <v>QA Engineer</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F106"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add project names to heatmap cells and fix revenue calculation
- Added project tags (short codes) to Resource Utilization Forecast heatmap
- Each cell now shows allocation % plus project abbreviations with tooltips
- Active projects shown in green, Planned in blue
- Fixed projected revenue calculation: CostRate × AllocationPercent × HoursPerWeek × 4.33
- Simplified data structure: removed Budget from Projects, Department from Resources
</commit_message>
<xml_diff>
--- a/resource_planning_data.xlsx
+++ b/resource_planning_data.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,15 +415,12 @@
         <v>SecondarySkill</v>
       </c>
       <c r="E1" t="str">
-        <v>Department</v>
+        <v>Status</v>
       </c>
       <c r="F1" t="str">
-        <v>Status</v>
+        <v>HoursPerWeek</v>
       </c>
       <c r="G1" t="str">
-        <v>HoursPerWeek</v>
-      </c>
-      <c r="H1" t="str">
         <v>CostRate</v>
       </c>
     </row>
@@ -441,15 +438,12 @@
         <v>UI/UX</v>
       </c>
       <c r="E2" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F2" t="str">
         <v>Active</v>
       </c>
+      <c r="F2">
+        <v>40</v>
+      </c>
       <c r="G2">
-        <v>40</v>
-      </c>
-      <c r="H2">
         <v>150</v>
       </c>
     </row>
@@ -467,15 +461,12 @@
         <v>DevOps</v>
       </c>
       <c r="E3" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F3" t="str">
         <v>Active</v>
       </c>
+      <c r="F3">
+        <v>40</v>
+      </c>
       <c r="G3">
-        <v>40</v>
-      </c>
-      <c r="H3">
         <v>160</v>
       </c>
     </row>
@@ -493,15 +484,12 @@
         <v>Python</v>
       </c>
       <c r="E4" t="str">
-        <v>Analytics</v>
-      </c>
-      <c r="F4" t="str">
         <v>Active</v>
       </c>
+      <c r="F4">
+        <v>40</v>
+      </c>
       <c r="G4">
-        <v>40</v>
-      </c>
-      <c r="H4">
         <v>175</v>
       </c>
     </row>
@@ -519,15 +507,12 @@
         <v>Agile</v>
       </c>
       <c r="E5" t="str">
-        <v>PMO</v>
-      </c>
-      <c r="F5" t="str">
         <v>Active</v>
       </c>
+      <c r="F5">
+        <v>40</v>
+      </c>
       <c r="G5">
-        <v>40</v>
-      </c>
-      <c r="H5">
         <v>140</v>
       </c>
     </row>
@@ -545,15 +530,12 @@
         <v>Database</v>
       </c>
       <c r="E6" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F6" t="str">
         <v>Active</v>
       </c>
+      <c r="F6">
+        <v>40</v>
+      </c>
       <c r="G6">
-        <v>40</v>
-      </c>
-      <c r="H6">
         <v>155</v>
       </c>
     </row>
@@ -571,15 +553,12 @@
         <v>React</v>
       </c>
       <c r="E7" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F7" t="str">
         <v>Active</v>
       </c>
+      <c r="F7">
+        <v>40</v>
+      </c>
       <c r="G7">
-        <v>40</v>
-      </c>
-      <c r="H7">
         <v>145</v>
       </c>
     </row>
@@ -597,15 +576,12 @@
         <v>Cloud</v>
       </c>
       <c r="E8" t="str">
-        <v>Infrastructure</v>
-      </c>
-      <c r="F8" t="str">
         <v>Active</v>
       </c>
+      <c r="F8">
+        <v>40</v>
+      </c>
       <c r="G8">
-        <v>40</v>
-      </c>
-      <c r="H8">
         <v>165</v>
       </c>
     </row>
@@ -623,15 +599,12 @@
         <v>Automation</v>
       </c>
       <c r="E9" t="str">
-        <v>Quality</v>
-      </c>
-      <c r="F9" t="str">
         <v>Active</v>
       </c>
+      <c r="F9">
+        <v>40</v>
+      </c>
       <c r="G9">
-        <v>40</v>
-      </c>
-      <c r="H9">
         <v>130</v>
       </c>
     </row>
@@ -649,15 +622,12 @@
         <v>Design</v>
       </c>
       <c r="E10" t="str">
-        <v>Design</v>
-      </c>
-      <c r="F10" t="str">
         <v>Active</v>
       </c>
+      <c r="F10">
+        <v>40</v>
+      </c>
       <c r="G10">
-        <v>40</v>
-      </c>
-      <c r="H10">
         <v>140</v>
       </c>
     </row>
@@ -675,15 +645,12 @@
         <v>ML</v>
       </c>
       <c r="E11" t="str">
-        <v>Analytics</v>
-      </c>
-      <c r="F11" t="str">
         <v>Active</v>
       </c>
+      <c r="F11">
+        <v>40</v>
+      </c>
       <c r="G11">
-        <v>40</v>
-      </c>
-      <c r="H11">
         <v>180</v>
       </c>
     </row>
@@ -701,15 +668,12 @@
         <v>API</v>
       </c>
       <c r="E12" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F12" t="str">
         <v>Active</v>
       </c>
+      <c r="F12">
+        <v>40</v>
+      </c>
       <c r="G12">
-        <v>40</v>
-      </c>
-      <c r="H12">
         <v>150</v>
       </c>
     </row>
@@ -727,15 +691,12 @@
         <v>Vue</v>
       </c>
       <c r="E13" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F13" t="str">
         <v>Active</v>
       </c>
+      <c r="F13">
+        <v>40</v>
+      </c>
       <c r="G13">
-        <v>40</v>
-      </c>
-      <c r="H13">
         <v>145</v>
       </c>
     </row>
@@ -753,15 +714,12 @@
         <v>Microservices</v>
       </c>
       <c r="E14" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="F14" t="str">
         <v>Active</v>
       </c>
+      <c r="F14">
+        <v>40</v>
+      </c>
       <c r="G14">
-        <v>40</v>
-      </c>
-      <c r="H14">
         <v>160</v>
       </c>
     </row>
@@ -779,15 +737,12 @@
         <v>Kubernetes</v>
       </c>
       <c r="E15" t="str">
-        <v>Infrastructure</v>
-      </c>
-      <c r="F15" t="str">
         <v>Active</v>
       </c>
+      <c r="F15">
+        <v>40</v>
+      </c>
       <c r="G15">
-        <v>40</v>
-      </c>
-      <c r="H15">
         <v>170</v>
       </c>
     </row>
@@ -805,28 +760,25 @@
         <v>Performance</v>
       </c>
       <c r="E16" t="str">
-        <v>Quality</v>
-      </c>
-      <c r="F16" t="str">
         <v>Active</v>
       </c>
+      <c r="F16">
+        <v>40</v>
+      </c>
       <c r="G16">
-        <v>40</v>
-      </c>
-      <c r="H16">
         <v>135</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:I12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -854,9 +806,6 @@
         <v>EndDate</v>
       </c>
       <c r="I1" t="str">
-        <v>Budget</v>
-      </c>
-      <c r="J1" t="str">
         <v>RequiredFTE</v>
       </c>
     </row>
@@ -886,9 +835,6 @@
         <v>2025-06-30</v>
       </c>
       <c r="I2">
-        <v>150000</v>
-      </c>
-      <c r="J2">
         <v>4</v>
       </c>
     </row>
@@ -918,9 +864,6 @@
         <v>2025-08-31</v>
       </c>
       <c r="I3">
-        <v>200000</v>
-      </c>
-      <c r="J3">
         <v>5</v>
       </c>
     </row>
@@ -950,9 +893,6 @@
         <v>2025-05-31</v>
       </c>
       <c r="I4">
-        <v>120000</v>
-      </c>
-      <c r="J4">
         <v>3</v>
       </c>
     </row>
@@ -982,9 +922,6 @@
         <v>2025-06-30</v>
       </c>
       <c r="I5">
-        <v>60000</v>
-      </c>
-      <c r="J5">
         <v>2</v>
       </c>
     </row>
@@ -1014,9 +951,6 @@
         <v>2025-08-15</v>
       </c>
       <c r="I6">
-        <v>80000</v>
-      </c>
-      <c r="J6">
         <v>3</v>
       </c>
     </row>
@@ -1046,9 +980,6 @@
         <v>2025-10-31</v>
       </c>
       <c r="I7">
-        <v>250000</v>
-      </c>
-      <c r="J7">
         <v>4</v>
       </c>
     </row>
@@ -1078,9 +1009,6 @@
         <v>2025-11-30</v>
       </c>
       <c r="I8">
-        <v>180000</v>
-      </c>
-      <c r="J8">
         <v>4</v>
       </c>
     </row>
@@ -1110,9 +1038,6 @@
         <v>2025-07-31</v>
       </c>
       <c r="I9">
-        <v>90000</v>
-      </c>
-      <c r="J9">
         <v>2</v>
       </c>
     </row>
@@ -1142,9 +1067,6 @@
         <v>2025-09-30</v>
       </c>
       <c r="I10">
-        <v>140000</v>
-      </c>
-      <c r="J10">
         <v>3</v>
       </c>
     </row>
@@ -1174,9 +1096,6 @@
         <v>2025-12-31</v>
       </c>
       <c r="I11">
-        <v>100000</v>
-      </c>
-      <c r="J11">
         <v>3</v>
       </c>
     </row>
@@ -1206,15 +1125,12 @@
         <v>2026-01-31</v>
       </c>
       <c r="I12">
-        <v>200000</v>
-      </c>
-      <c r="J12">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>